<commit_message>
update: 2026/06/22 周一 13:27:24.96
</commit_message>
<xml_diff>
--- a/source/7、连续未出勤/未出勤工伤剔除-5月.xlsx
+++ b/source/7、连续未出勤/未出勤工伤剔除-5月.xlsx
@@ -10,7 +10,7 @@
     <sheet name="4月" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'4月'!$A$1:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'4月'!$A$1:$G$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,12 +29,8 @@
 </workbook>
 </file>
 
-<file path=xl/cellimages.xml><?xml version="1.0" encoding="utf-8"?>
-<etc:cellImages xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData"/>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
   <si>
     <t>工号</t>
   </si>
@@ -103,9 +99,6 @@
   </si>
   <si>
     <t>李玉友</t>
-  </si>
-  <si>
-    <t>浙北区</t>
   </si>
 </sst>
 </file>
@@ -1204,7 +1197,7 @@
         <v>22</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
@@ -1217,7 +1210,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G2" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G5" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>